<commit_message>
working version before API integration
</commit_message>
<xml_diff>
--- a/combine_data.xlsx
+++ b/combine_data.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54e5b2c583474f06/Documentos/safe-to-swim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_6C01B0A0D3D05C29E513D8734B5ED87656C170CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B878C19D-6E1C-4828-8E68-5589BFC80E9F}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_6C01B0A0D3D05C29E513D8734B5ED87656C170CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4362D873-BBA0-4F2F-8585-E66A5D9893E8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -2241,7 +2244,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -2274,7 +2277,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2290,6 +2293,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2580,7 +2587,9 @@
   <dimension ref="A1:T1001"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
     <col min="10" max="10" width="13.44140625" customWidth="1"/>
+    <col min="15" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
@@ -58637,6 +58646,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:T1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>